<commit_message>
Demo neutra per gli screenshot pubblici
Catalogo sintetico multi-marca e multi-categoria (cura della persona,
igiene, piccoli elettrodomestici) al posto di quello del settore reale.
Ogni fornitore applica il proprio scostamento su un prezzo di riferimento,
e tre articoli esistono anche come gemelli OEM a marchio del grossista,
con EAN diverso e prezzo più basso. Template e script di carico neutri.

Benchmark visivo rifatto sul nuovo set (SigLIP 2, sintetico): R@5 92,9%
a foto intera, 100% con ritaglio. Decisione D-022.
</commit_message>
<xml_diff>
--- a/fixtures/demo/beta-wholesale.xlsx
+++ b/fixtures/demo/beta-wholesale.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="238" uniqueCount="151">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="258" uniqueCount="165">
   <si>
     <t>Item No</t>
   </si>
@@ -52,19 +52,19 @@
     <t>Product URL</t>
   </si>
   <si>
-    <t>BW-P001-50ML</t>
+    <t>BW-P001-250ML</t>
   </si>
   <si>
     <t>8009900000013</t>
   </si>
   <si>
-    <t>Lumen Care Gel Idratante 50 ml (blu)</t>
-  </si>
-  <si>
-    <t>Lumen Care Srl</t>
-  </si>
-  <si>
-    <t>Lubes</t>
+    <t>Solvetta Shampoo Nutriente 250 ml (blu)</t>
+  </si>
+  <si>
+    <t>Solvetta Srl</t>
+  </si>
+  <si>
+    <t>Hair care</t>
   </si>
   <si>
     <t>Blu</t>
@@ -79,19 +79,19 @@
     <t>http://127.0.0.1:4010/beta-p001.jpg</t>
   </si>
   <si>
-    <t>https://beta.example.com/item/p001-50ml</t>
-  </si>
-  <si>
-    <t>BW-P001-100ML</t>
+    <t>https://beta.example.com/item/p001-250ml</t>
+  </si>
+  <si>
+    <t>BW-P001-500ML</t>
   </si>
   <si>
     <t>8009900000020</t>
   </si>
   <si>
-    <t>Lumen Care Gel Idratante 100 ml (blu)</t>
-  </si>
-  <si>
-    <t>Lumen Care</t>
+    <t>Solvetta Shampoo Nutriente 500 ml (blu)</t>
+  </si>
+  <si>
+    <t>Solvetta</t>
   </si>
   <si>
     <t>Low stock</t>
@@ -100,19 +100,19 @@
     <t>1 week</t>
   </si>
   <si>
-    <t>https://beta.example.com/item/p001-100ml</t>
-  </si>
-  <si>
-    <t>BW-P002-100ML</t>
+    <t>https://beta.example.com/item/p001-500ml</t>
+  </si>
+  <si>
+    <t>BW-P002-500ML</t>
   </si>
   <si>
     <t>8009900000044</t>
   </si>
   <si>
-    <t>Sensa Lubrificante Acqua 100 ml (oro)</t>
-  </si>
-  <si>
-    <t>Sensa</t>
+    <t>Marvessa Shampoo Delicato 500 ml (oro)</t>
+  </si>
+  <si>
+    <t>Marvessa</t>
   </si>
   <si>
     <t>Oro</t>
@@ -127,234 +127,237 @@
     <t>http://127.0.0.1:4010/beta-p002.jpg</t>
   </si>
   <si>
-    <t>https://beta.example.com/item/p002-100ml</t>
-  </si>
-  <si>
-    <t>BW-P003-50ML</t>
-  </si>
-  <si>
-    <t>Moira Silk Gel 50 ml (fucsia)</t>
-  </si>
-  <si>
-    <t>Moira</t>
+    <t>https://beta.example.com/item/p002-500ml</t>
+  </si>
+  <si>
+    <t>BW-P003-250ML</t>
+  </si>
+  <si>
+    <t>Marvessa Balsamo Lisciante 250 ml (nero)</t>
+  </si>
+  <si>
+    <t>Nero</t>
+  </si>
+  <si>
+    <t>48h</t>
+  </si>
+  <si>
+    <t>http://127.0.0.1:4010/beta-p003.jpg</t>
+  </si>
+  <si>
+    <t>https://beta.example.com/item/p003-250ml</t>
+  </si>
+  <si>
+    <t>BW-P004-250ML</t>
+  </si>
+  <si>
+    <t>8009900000075</t>
+  </si>
+  <si>
+    <t>Olvari Olio Capelli 250 ml (rosa cipria)</t>
+  </si>
+  <si>
+    <t>Olvari Srl</t>
+  </si>
+  <si>
+    <t>Rosa cipria</t>
+  </si>
+  <si>
+    <t>Available</t>
+  </si>
+  <si>
+    <t>http://127.0.0.1:4010/beta-p004.jpg</t>
+  </si>
+  <si>
+    <t>https://beta.example.com/item/p004-250ml</t>
+  </si>
+  <si>
+    <t>BW-P004-500ML</t>
+  </si>
+  <si>
+    <t>8009900000082</t>
+  </si>
+  <si>
+    <t>Olvari Olio Capelli 500 ml (rosa cipria)</t>
+  </si>
+  <si>
+    <t>Olvari</t>
+  </si>
+  <si>
+    <t>On order</t>
+  </si>
+  <si>
+    <t>https://beta.example.com/item/p004-500ml</t>
+  </si>
+  <si>
+    <t>BW-P006-75ML</t>
+  </si>
+  <si>
+    <t>8009900000105</t>
+  </si>
+  <si>
+    <t>Olvari Crema Viso Idratante 75 ml (oro)</t>
+  </si>
+  <si>
+    <t>Body care</t>
+  </si>
+  <si>
+    <t>http://127.0.0.1:4010/beta-p006.jpg</t>
+  </si>
+  <si>
+    <t>https://beta.example.com/item/p006-75ml</t>
+  </si>
+  <si>
+    <t>BW-P007-75ML</t>
+  </si>
+  <si>
+    <t>Brivanto Gel Doccia Agrumi 75 ml (nero)</t>
+  </si>
+  <si>
+    <t>Brivanto</t>
+  </si>
+  <si>
+    <t>http://127.0.0.1:4010/beta-p007.jpg</t>
+  </si>
+  <si>
+    <t>https://beta.example.com/item/p007-75ml</t>
+  </si>
+  <si>
+    <t>BW-P009-20PZ</t>
+  </si>
+  <si>
+    <t>8009900000136</t>
+  </si>
+  <si>
+    <t>Solvetta Salviette Struccanti 20 pz (oro)</t>
+  </si>
+  <si>
+    <t>Hygiene</t>
+  </si>
+  <si>
+    <t>http://127.0.0.1:4010/beta-p009.jpg</t>
+  </si>
+  <si>
+    <t>https://beta.example.com/item/p009-20pz</t>
+  </si>
+  <si>
+    <t>BW-P010-20PZ</t>
+  </si>
+  <si>
+    <t>8009900000143</t>
+  </si>
+  <si>
+    <t>Quellora Cerotti Delicati 20 pz (rosa cipria)</t>
+  </si>
+  <si>
+    <t>Quellora</t>
+  </si>
+  <si>
+    <t>http://127.0.0.1:4010/beta-p010.jpg</t>
+  </si>
+  <si>
+    <t>https://beta.example.com/item/p010-20pz</t>
+  </si>
+  <si>
+    <t>BW-P012-STANDARD</t>
+  </si>
+  <si>
+    <t>8009900000167</t>
+  </si>
+  <si>
+    <t>Olvari Asciugacapelli Pro Standard (rosa cipria)</t>
+  </si>
+  <si>
+    <t>Small appliances</t>
+  </si>
+  <si>
+    <t>http://127.0.0.1:4010/beta-p012.jpg</t>
+  </si>
+  <si>
+    <t>https://beta.example.com/item/p012-Standard</t>
+  </si>
+  <si>
+    <t>BW-P013-STANDARD</t>
+  </si>
+  <si>
+    <t>8009900000174</t>
+  </si>
+  <si>
+    <t>Olvari Asciugacapelli Pro Standard (verde)</t>
+  </si>
+  <si>
+    <t>Verde</t>
+  </si>
+  <si>
+    <t>http://127.0.0.1:4010/beta-p013.jpg</t>
+  </si>
+  <si>
+    <t>https://beta.example.com/item/p013-Standard</t>
+  </si>
+  <si>
+    <t>BW-P015-STANDARD</t>
+  </si>
+  <si>
+    <t>8009900000198</t>
+  </si>
+  <si>
+    <t>Tessavo Asciugacapelli Compact Standard (fucsia)</t>
+  </si>
+  <si>
+    <t>Tessavo Srl</t>
   </si>
   <si>
     <t>Fucsia</t>
   </si>
   <si>
-    <t>48h</t>
-  </si>
-  <si>
-    <t>http://127.0.0.1:4010/beta-p003.jpg</t>
-  </si>
-  <si>
-    <t>https://beta.example.com/item/p003-50ml</t>
-  </si>
-  <si>
-    <t>BW-P004-50ML</t>
-  </si>
-  <si>
-    <t>8009900000075</t>
-  </si>
-  <si>
-    <t>Moira Olio Massaggio 50 ml (nero)</t>
-  </si>
-  <si>
-    <t>Moira Srl</t>
-  </si>
-  <si>
-    <t>Nero</t>
-  </si>
-  <si>
-    <t>Available</t>
-  </si>
-  <si>
-    <t>http://127.0.0.1:4010/beta-p004.jpg</t>
-  </si>
-  <si>
-    <t>https://beta.example.com/item/p004-50ml</t>
-  </si>
-  <si>
-    <t>BW-P004-100ML</t>
-  </si>
-  <si>
-    <t>8009900000082</t>
-  </si>
-  <si>
-    <t>Moira Olio Massaggio 100 ml (nero)</t>
-  </si>
-  <si>
-    <t>On order</t>
-  </si>
-  <si>
-    <t>https://beta.example.com/item/p004-100ml</t>
-  </si>
-  <si>
-    <t>BW-P006-30ML</t>
-  </si>
-  <si>
-    <t>8009900000105</t>
-  </si>
-  <si>
-    <t>Aurum Balsamo Relax 30 ml (fucsia)</t>
-  </si>
-  <si>
-    <t>Aurum</t>
-  </si>
-  <si>
-    <t>Wellness</t>
-  </si>
-  <si>
-    <t>http://127.0.0.1:4010/beta-p006.jpg</t>
-  </si>
-  <si>
-    <t>https://beta.example.com/item/p006-30ml</t>
-  </si>
-  <si>
-    <t>BW-P007-30ML</t>
-  </si>
-  <si>
-    <t>Lumen Care Gel Calore 30 ml (rosa cipria)</t>
-  </si>
-  <si>
-    <t>Rosa cipria</t>
-  </si>
-  <si>
-    <t>http://127.0.0.1:4010/beta-p007.jpg</t>
-  </si>
-  <si>
-    <t>https://beta.example.com/item/p007-30ml</t>
-  </si>
-  <si>
-    <t>BW-P009-6PZ</t>
-  </si>
-  <si>
-    <t>8009900000136</t>
-  </si>
-  <si>
-    <t>Moira Classic 6 pz (fucsia)</t>
-  </si>
-  <si>
-    <t>Condoms</t>
-  </si>
-  <si>
-    <t>http://127.0.0.1:4010/beta-p009.jpg</t>
-  </si>
-  <si>
-    <t>https://beta.example.com/item/p009-6pz</t>
-  </si>
-  <si>
-    <t>BW-P010-6PZ</t>
-  </si>
-  <si>
-    <t>8009900000143</t>
-  </si>
-  <si>
-    <t>Nuvia Extra Large 6 pz (nero)</t>
-  </si>
-  <si>
-    <t>Nuvia</t>
-  </si>
-  <si>
-    <t>http://127.0.0.1:4010/beta-p010.jpg</t>
-  </si>
-  <si>
-    <t>https://beta.example.com/item/p010-6pz</t>
-  </si>
-  <si>
-    <t>BW-P012-STANDARD</t>
-  </si>
-  <si>
-    <t>8009900000167</t>
-  </si>
-  <si>
-    <t>Sensa Wave Standard (viola)</t>
-  </si>
-  <si>
-    <t>Toys</t>
+    <t>http://127.0.0.1:4010/beta-p015.jpg</t>
+  </si>
+  <si>
+    <t>https://beta.example.com/item/p015-Standard</t>
+  </si>
+  <si>
+    <t>BW-P016-STANDARD</t>
+  </si>
+  <si>
+    <t>8009900000204</t>
+  </si>
+  <si>
+    <t>Olvari Asciugacapelli Ionico Standard (blu)</t>
+  </si>
+  <si>
+    <t>http://127.0.0.1:4010/beta-p016.jpg</t>
+  </si>
+  <si>
+    <t>https://beta.example.com/item/p016-Standard</t>
+  </si>
+  <si>
+    <t>BW-P018-STANDARD</t>
+  </si>
+  <si>
+    <t>8009900000228</t>
+  </si>
+  <si>
+    <t>Olvari Asciugacapelli Travel Standard (fucsia)</t>
+  </si>
+  <si>
+    <t>http://127.0.0.1:4010/beta-p018.jpg</t>
+  </si>
+  <si>
+    <t>https://beta.example.com/item/p018-Standard</t>
+  </si>
+  <si>
+    <t>BW-P019-STANDARD</t>
+  </si>
+  <si>
+    <t>8009900000235</t>
+  </si>
+  <si>
+    <t>Olvari Asciugacapelli Travel Standard (viola)</t>
   </si>
   <si>
     <t>Viola</t>
   </si>
   <si>
-    <t>http://127.0.0.1:4010/beta-p012.jpg</t>
-  </si>
-  <si>
-    <t>https://beta.example.com/item/p012-Standard</t>
-  </si>
-  <si>
-    <t>BW-P013-STANDARD</t>
-  </si>
-  <si>
-    <t>8009900000174</t>
-  </si>
-  <si>
-    <t>Sensa Wave Standard (nero)</t>
-  </si>
-  <si>
-    <t>http://127.0.0.1:4010/beta-p013.jpg</t>
-  </si>
-  <si>
-    <t>https://beta.example.com/item/p013-Standard</t>
-  </si>
-  <si>
-    <t>BW-P015-STANDARD</t>
-  </si>
-  <si>
-    <t>8009900000198</t>
-  </si>
-  <si>
-    <t>Moira Orbit Standard (fucsia)</t>
-  </si>
-  <si>
-    <t>http://127.0.0.1:4010/beta-p015.jpg</t>
-  </si>
-  <si>
-    <t>https://beta.example.com/item/p015-Standard</t>
-  </si>
-  <si>
-    <t>BW-P016-STANDARD</t>
-  </si>
-  <si>
-    <t>8009900000204</t>
-  </si>
-  <si>
-    <t>Aurum Petal Standard (rosa cipria)</t>
-  </si>
-  <si>
-    <t>http://127.0.0.1:4010/beta-p016.jpg</t>
-  </si>
-  <si>
-    <t>https://beta.example.com/item/p016-Standard</t>
-  </si>
-  <si>
-    <t>BW-P018-STANDARD</t>
-  </si>
-  <si>
-    <t>8009900000228</t>
-  </si>
-  <si>
-    <t>Lumen Care Curve Standard (verde)</t>
-  </si>
-  <si>
-    <t>Verde</t>
-  </si>
-  <si>
-    <t>http://127.0.0.1:4010/beta-p018.jpg</t>
-  </si>
-  <si>
-    <t>https://beta.example.com/item/p018-Standard</t>
-  </si>
-  <si>
-    <t>BW-P019-STANDARD</t>
-  </si>
-  <si>
-    <t>8009900000235</t>
-  </si>
-  <si>
-    <t>Lumen Care Curve Standard (oro)</t>
-  </si>
-  <si>
     <t>http://127.0.0.1:4010/beta-p019.jpg</t>
   </si>
   <si>
@@ -367,10 +370,10 @@
     <t>8009900000259</t>
   </si>
   <si>
-    <t>Aurum Slim Classic Standard (verde)</t>
-  </si>
-  <si>
-    <t>Aurum Srl</t>
+    <t>Marvessa Spazzolino Sonico Standard (verde)</t>
+  </si>
+  <si>
+    <t>Marvessa Srl</t>
   </si>
   <si>
     <t>http://127.0.0.1:4010/beta-p021.jpg</t>
@@ -385,7 +388,7 @@
     <t>8009900000266</t>
   </si>
   <si>
-    <t>Aurum Bullet Standard (rosa cipria)</t>
+    <t>Marvessa Spazzolino Ricaricabile Standard (verde)</t>
   </si>
   <si>
     <t>http://127.0.0.1:4010/beta-p022.jpg</t>
@@ -400,7 +403,7 @@
     <t>8009900000280</t>
   </si>
   <si>
-    <t>Lumen Care Wand Mini Standard (fucsia)</t>
+    <t>Solvetta Spazzolino Junior Standard (oro)</t>
   </si>
   <si>
     <t>http://127.0.0.1:4010/beta-p024.jpg</t>
@@ -415,7 +418,7 @@
     <t>8009900000297</t>
   </si>
   <si>
-    <t>Lumen Care Wand Mini Standard (viola)</t>
+    <t>Solvetta Spazzolino Junior Standard (nero)</t>
   </si>
   <si>
     <t>http://127.0.0.1:4010/beta-p025.jpg</t>
@@ -430,7 +433,7 @@
     <t>8009900000310</t>
   </si>
   <si>
-    <t>Moira Scrub Sensuale 200 ml (verde)</t>
+    <t>Marvessa Scrub Corpo 200 ml (fucsia)</t>
   </si>
   <si>
     <t>http://127.0.0.1:4010/beta-p027.jpg</t>
@@ -445,7 +448,13 @@
     <t>8009900000327</t>
   </si>
   <si>
-    <t>Sensa Anello Flex Standard (verde)</t>
+    <t>Tessavo Elastici Spirale Standard (nero)</t>
+  </si>
+  <si>
+    <t>Tessavo</t>
+  </si>
+  <si>
+    <t>Hair accessories</t>
   </si>
   <si>
     <t>http://127.0.0.1:4010/beta-p028.jpg</t>
@@ -457,13 +466,46 @@
     <t>BW-CONFLICT-1</t>
   </si>
   <si>
-    <t>Massager Wave (other brand)</t>
+    <t>Hair Dryer Pro (other brand)</t>
   </si>
   <si>
     <t>OtherBrand</t>
   </si>
   <si>
     <t>Giallo</t>
+  </si>
+  <si>
+    <t>BW-OWN-T01</t>
+  </si>
+  <si>
+    <t>8009900000341</t>
+  </si>
+  <si>
+    <t>Beta Essentials Asciugacapelli 2200W Standard (verde)</t>
+  </si>
+  <si>
+    <t>Beta Essentials</t>
+  </si>
+  <si>
+    <t>http://127.0.0.1:4010/beta-t01.jpg</t>
+  </si>
+  <si>
+    <t>https://beta.example.com/item/t01</t>
+  </si>
+  <si>
+    <t>BW-OWN-T02</t>
+  </si>
+  <si>
+    <t>8009900000358</t>
+  </si>
+  <si>
+    <t>Beta Essentials Balsamo Capelli Lisci 250 ml (nero)</t>
+  </si>
+  <si>
+    <t>http://127.0.0.1:4010/beta-t02.jpg</t>
+  </si>
+  <si>
+    <t>https://beta.example.com/item/t02</t>
   </si>
 </sst>
 </file>
@@ -841,7 +883,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:M24"/>
+  <dimension ref="A1:M26"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.25">
@@ -905,7 +947,7 @@
         <v>18</v>
       </c>
       <c r="G2">
-        <v>23.92</v>
+        <v>7.07</v>
       </c>
       <c r="H2">
         <v>1</v>
@@ -946,7 +988,7 @@
         <v>18</v>
       </c>
       <c r="G3">
-        <v>7.28</v>
+        <v>11.69</v>
       </c>
       <c r="H3">
         <v>1</v>
@@ -984,7 +1026,7 @@
         <v>34</v>
       </c>
       <c r="G4">
-        <v>22.52</v>
+        <v>6.86</v>
       </c>
       <c r="H4">
         <v>1</v>
@@ -1013,16 +1055,16 @@
         <v>40</v>
       </c>
       <c r="D5" t="s">
-        <v>41</v>
+        <v>33</v>
       </c>
       <c r="E5" t="s">
         <v>17</v>
       </c>
       <c r="F5" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="G5">
-        <v>28.55</v>
+        <v>10.36</v>
       </c>
       <c r="H5">
         <v>1</v>
@@ -1031,74 +1073,74 @@
         <v>19</v>
       </c>
       <c r="K5" t="s">
+        <v>42</v>
+      </c>
+      <c r="L5" t="s">
         <v>43</v>
       </c>
-      <c r="L5" t="s">
+      <c r="M5" t="s">
         <v>44</v>
-      </c>
-      <c r="M5" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>45</v>
+      </c>
+      <c r="B6" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="C6" t="s">
         <v>47</v>
       </c>
-      <c r="C6" t="s">
+      <c r="D6" t="s">
         <v>48</v>
-      </c>
-      <c r="D6" t="s">
-        <v>49</v>
       </c>
       <c r="E6" t="s">
         <v>17</v>
       </c>
       <c r="F6" t="s">
+        <v>49</v>
+      </c>
+      <c r="G6">
+        <v>3.29</v>
+      </c>
+      <c r="H6">
+        <v>1</v>
+      </c>
+      <c r="J6" t="s">
         <v>50</v>
-      </c>
-      <c r="G6">
-        <v>5.45</v>
-      </c>
-      <c r="H6">
-        <v>1</v>
-      </c>
-      <c r="J6" t="s">
-        <v>51</v>
       </c>
       <c r="K6" t="s">
         <v>20</v>
       </c>
       <c r="L6" t="s">
+        <v>51</v>
+      </c>
+      <c r="M6" t="s">
         <v>52</v>
-      </c>
-      <c r="M6" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>53</v>
+      </c>
+      <c r="B7" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="C7" t="s">
         <v>55</v>
       </c>
-      <c r="C7" t="s">
+      <c r="D7" t="s">
         <v>56</v>
-      </c>
-      <c r="D7" t="s">
-        <v>41</v>
       </c>
       <c r="E7" t="s">
         <v>17</v>
       </c>
       <c r="F7" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="G7">
-        <v>10.73</v>
+        <v>6.36</v>
       </c>
       <c r="H7">
         <v>1</v>
@@ -1113,7 +1155,7 @@
         <v>28</v>
       </c>
       <c r="L7" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="M7" t="s">
         <v>58</v>
@@ -1130,16 +1172,16 @@
         <v>61</v>
       </c>
       <c r="D8" t="s">
+        <v>56</v>
+      </c>
+      <c r="E8" t="s">
         <v>62</v>
       </c>
-      <c r="E8" t="s">
-        <v>63</v>
-      </c>
       <c r="F8" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="G8">
-        <v>14.52</v>
+        <v>4.34</v>
       </c>
       <c r="H8">
         <v>1</v>
@@ -1151,33 +1193,33 @@
         <v>36</v>
       </c>
       <c r="L8" t="s">
+        <v>63</v>
+      </c>
+      <c r="M8" t="s">
         <v>64</v>
-      </c>
-      <c r="M8" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B9">
         <v>8009900000112</v>
       </c>
       <c r="C9" t="s">
+        <v>66</v>
+      </c>
+      <c r="D9" t="s">
         <v>67</v>
       </c>
-      <c r="D9" t="s">
-        <v>26</v>
-      </c>
       <c r="E9" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F9" t="s">
-        <v>68</v>
+        <v>41</v>
       </c>
       <c r="G9">
-        <v>10.93</v>
+        <v>7.38</v>
       </c>
       <c r="H9">
         <v>1</v>
@@ -1186,33 +1228,33 @@
         <v>27</v>
       </c>
       <c r="K9" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="L9" t="s">
+        <v>68</v>
+      </c>
+      <c r="M9" t="s">
         <v>69</v>
-      </c>
-      <c r="M9" t="s">
-        <v>70</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>70</v>
+      </c>
+      <c r="B10" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="C10" t="s">
         <v>72</v>
       </c>
-      <c r="C10" t="s">
+      <c r="D10" t="s">
+        <v>16</v>
+      </c>
+      <c r="E10" t="s">
         <v>73</v>
       </c>
-      <c r="D10" t="s">
-        <v>49</v>
-      </c>
-      <c r="E10" t="s">
-        <v>74</v>
-      </c>
       <c r="G10">
-        <v>34.25</v>
+        <v>34.16</v>
       </c>
       <c r="H10">
         <v>5</v>
@@ -1224,30 +1266,30 @@
         <v>20</v>
       </c>
       <c r="L10" t="s">
+        <v>74</v>
+      </c>
+      <c r="M10" t="s">
         <v>75</v>
-      </c>
-      <c r="M10" t="s">
-        <v>76</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
+        <v>76</v>
+      </c>
+      <c r="B11" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="C11" t="s">
         <v>78</v>
       </c>
-      <c r="C11" t="s">
+      <c r="D11" t="s">
         <v>79</v>
       </c>
-      <c r="D11" t="s">
-        <v>80</v>
-      </c>
       <c r="E11" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="G11">
-        <v>20.7</v>
+        <v>29.05</v>
       </c>
       <c r="H11">
         <v>5</v>
@@ -1259,33 +1301,33 @@
         <v>28</v>
       </c>
       <c r="L11" t="s">
+        <v>80</v>
+      </c>
+      <c r="M11" t="s">
         <v>81</v>
-      </c>
-      <c r="M11" t="s">
-        <v>82</v>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
+        <v>82</v>
+      </c>
+      <c r="B12" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="B12" s="1" t="s">
+      <c r="C12" t="s">
         <v>84</v>
       </c>
-      <c r="C12" t="s">
+      <c r="D12" t="s">
+        <v>56</v>
+      </c>
+      <c r="E12" t="s">
         <v>85</v>
       </c>
-      <c r="D12" t="s">
-        <v>33</v>
-      </c>
-      <c r="E12" t="s">
-        <v>86</v>
-      </c>
       <c r="F12" t="s">
-        <v>87</v>
+        <v>49</v>
       </c>
       <c r="G12">
-        <v>25.06</v>
+        <v>18.06</v>
       </c>
       <c r="H12">
         <v>1</v>
@@ -1294,39 +1336,39 @@
         <v>3</v>
       </c>
       <c r="J12" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="K12" t="s">
         <v>36</v>
       </c>
       <c r="L12" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="M12" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
+        <v>88</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="C13" t="s">
         <v>90</v>
       </c>
-      <c r="B13" s="1" t="s">
+      <c r="D13" t="s">
+        <v>56</v>
+      </c>
+      <c r="E13" t="s">
+        <v>85</v>
+      </c>
+      <c r="F13" t="s">
         <v>91</v>
       </c>
-      <c r="C13" t="s">
-        <v>92</v>
-      </c>
-      <c r="D13" t="s">
-        <v>33</v>
-      </c>
-      <c r="E13" t="s">
-        <v>86</v>
-      </c>
-      <c r="F13" t="s">
-        <v>50</v>
-      </c>
       <c r="G13">
-        <v>20.42</v>
+        <v>43.07</v>
       </c>
       <c r="H13">
         <v>1</v>
@@ -1335,36 +1377,36 @@
         <v>57</v>
       </c>
       <c r="K13" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="L13" t="s">
+        <v>92</v>
+      </c>
+      <c r="M13" t="s">
         <v>93</v>
-      </c>
-      <c r="M13" t="s">
-        <v>94</v>
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
+        <v>94</v>
+      </c>
+      <c r="B14" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="B14" s="1" t="s">
+      <c r="C14" t="s">
         <v>96</v>
       </c>
-      <c r="C14" t="s">
+      <c r="D14" t="s">
         <v>97</v>
       </c>
-      <c r="D14" t="s">
-        <v>49</v>
-      </c>
       <c r="E14" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F14" t="s">
-        <v>42</v>
+        <v>98</v>
       </c>
       <c r="G14">
-        <v>15.34</v>
+        <v>21.83</v>
       </c>
       <c r="H14">
         <v>1</v>
@@ -1376,33 +1418,33 @@
         <v>20</v>
       </c>
       <c r="L14" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="M14" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C15" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D15" t="s">
-        <v>62</v>
+        <v>56</v>
       </c>
       <c r="E15" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F15" t="s">
-        <v>68</v>
+        <v>18</v>
       </c>
       <c r="G15">
-        <v>16.55</v>
+        <v>49.85</v>
       </c>
       <c r="H15">
         <v>1</v>
@@ -1414,33 +1456,33 @@
         <v>28</v>
       </c>
       <c r="L15" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="M15" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C16" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D16" t="s">
-        <v>26</v>
+        <v>56</v>
       </c>
       <c r="E16" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F16" t="s">
-        <v>108</v>
+        <v>98</v>
       </c>
       <c r="G16">
-        <v>5.58</v>
+        <v>31.74</v>
       </c>
       <c r="H16">
         <v>1</v>
@@ -1469,16 +1511,16 @@
         <v>113</v>
       </c>
       <c r="D17" t="s">
-        <v>26</v>
+        <v>56</v>
       </c>
       <c r="E17" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F17" t="s">
-        <v>34</v>
+        <v>114</v>
       </c>
       <c r="G17">
-        <v>6.79</v>
+        <v>37.22</v>
       </c>
       <c r="H17">
         <v>1</v>
@@ -1490,74 +1532,74 @@
         <v>19</v>
       </c>
       <c r="K17" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="L17" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="M17" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C18" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D18" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="E18" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F18" t="s">
-        <v>108</v>
+        <v>91</v>
       </c>
       <c r="G18">
-        <v>23.84</v>
+        <v>19.38</v>
       </c>
       <c r="H18">
         <v>1</v>
       </c>
       <c r="J18" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="K18" t="s">
         <v>20</v>
       </c>
       <c r="L18" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="M18" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C19" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D19" t="s">
-        <v>62</v>
+        <v>33</v>
       </c>
       <c r="E19" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F19" t="s">
-        <v>68</v>
+        <v>91</v>
       </c>
       <c r="G19">
-        <v>18.65</v>
+        <v>30.77</v>
       </c>
       <c r="H19">
         <v>1</v>
@@ -1569,33 +1611,33 @@
         <v>28</v>
       </c>
       <c r="L19" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="M19" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C20" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="D20" t="s">
         <v>26</v>
       </c>
       <c r="E20" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F20" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="G20">
-        <v>26.16</v>
+        <v>29.69</v>
       </c>
       <c r="H20">
         <v>1</v>
@@ -1607,33 +1649,33 @@
         <v>36</v>
       </c>
       <c r="L20" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="M20" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C21" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D21" t="s">
         <v>26</v>
       </c>
       <c r="E21" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F21" t="s">
-        <v>87</v>
+        <v>41</v>
       </c>
       <c r="G21">
-        <v>19.92</v>
+        <v>32.15</v>
       </c>
       <c r="H21">
         <v>1</v>
@@ -1642,36 +1684,36 @@
         <v>27</v>
       </c>
       <c r="K21" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="L21" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="M21" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C22" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="D22" t="s">
-        <v>49</v>
+        <v>120</v>
       </c>
       <c r="E22" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F22" t="s">
-        <v>108</v>
+        <v>98</v>
       </c>
       <c r="G22">
-        <v>10.9</v>
+        <v>6.81</v>
       </c>
       <c r="H22">
         <v>1</v>
@@ -1686,33 +1728,33 @@
         <v>20</v>
       </c>
       <c r="L22" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="M22" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C23" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="D23" t="s">
-        <v>33</v>
+        <v>146</v>
       </c>
       <c r="E23" t="s">
-        <v>63</v>
+        <v>147</v>
       </c>
       <c r="F23" t="s">
-        <v>108</v>
+        <v>41</v>
       </c>
       <c r="G23">
-        <v>29.29</v>
+        <v>2.48</v>
       </c>
       <c r="H23">
         <v>1</v>
@@ -1724,33 +1766,33 @@
         <v>28</v>
       </c>
       <c r="L23" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="M23" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="B24" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C24" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="D24" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="E24" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F24" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="G24">
-        <v>19.9</v>
+        <v>24.9</v>
       </c>
       <c r="H24">
         <v>1</v>
@@ -1762,7 +1804,83 @@
         <v>28</v>
       </c>
       <c r="L24" t="s">
-        <v>88</v>
+        <v>86</v>
+      </c>
+    </row>
+    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>154</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="C25" t="s">
+        <v>156</v>
+      </c>
+      <c r="D25" t="s">
+        <v>157</v>
+      </c>
+      <c r="E25" t="s">
+        <v>85</v>
+      </c>
+      <c r="F25" t="s">
+        <v>91</v>
+      </c>
+      <c r="G25">
+        <v>34.08</v>
+      </c>
+      <c r="H25">
+        <v>1</v>
+      </c>
+      <c r="J25" t="s">
+        <v>19</v>
+      </c>
+      <c r="K25" t="s">
+        <v>42</v>
+      </c>
+      <c r="L25" t="s">
+        <v>158</v>
+      </c>
+      <c r="M25" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>160</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="C26" t="s">
+        <v>162</v>
+      </c>
+      <c r="D26" t="s">
+        <v>157</v>
+      </c>
+      <c r="E26" t="s">
+        <v>17</v>
+      </c>
+      <c r="F26" t="s">
+        <v>41</v>
+      </c>
+      <c r="G26">
+        <v>7.47</v>
+      </c>
+      <c r="H26">
+        <v>1</v>
+      </c>
+      <c r="J26" t="s">
+        <v>19</v>
+      </c>
+      <c r="K26" t="s">
+        <v>42</v>
+      </c>
+      <c r="L26" t="s">
+        <v>163</v>
+      </c>
+      <c r="M26" t="s">
+        <v>164</v>
       </c>
     </row>
   </sheetData>

</xml_diff>